<commit_message>
Heladería EN, revisión D203: entregables remontados, gates en verde y REVISION-FINAL (0 B · 5 M · 12 m)
Remontado en el VPS: G1-G9 VERDE, autotests 20/20 y 8/8, barrido 1,383 piezas sin fallos, regresión 31/31 IGUAL,
2.ª pasada con sha256 canónico igual, Word de 24 págs. Letter. Volcados de revision/ regenerados.

Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/ice-cream-shop-business-plan/ice-cream-shop-financial-projections.xlsx
+++ b/astro-site/public/dl/ice-cream-shop-business-plan/ice-cream-shop-financial-projections.xlsx
@@ -1062,7 +1062,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mostly electricity: about 30 kW of service, with the dipping cabinets running 24 hours a day, the batch freezer, the hardening cabinet and the air conditioning. Summer sends the bill up; ask the landlord or the utility for the local's history</t>
+          <t>Mostly electricity: about 30 kW of service, with the dipping cabinets running 24 hours a day, the batch freezer, the hardening cabinet and the air conditioning. Summer sends the bill up; ask the landlord or the utility for the space's billing history</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Example rate: state + local sales tax combined. It varies widely by state and city: look up yours. UK: 20% VAT on hot food and dine-in</t>
+          <t>Example rate: state + local sales tax combined. It varies widely by state and city: look up yours. UK: ice cream is standard-rated at 20% VAT, to take away too</t>
         </is>
       </c>
     </row>
@@ -2009,7 +2009,7 @@
       </c>
       <c r="D18" s="28" t="inlineStr">
         <is>
-          <t>Front counter, dipper wells with running water (Food Code 3-304.12), espresso machine and grinder, waffle cone irons and hot fudge warmers. No exhaust hood needed: waffle cone irons produce no smoke</t>
+          <t>Front counter, dipper wells with running water (Food Code 3-304.12), espresso machine and grinder, waffle cone irons and hot fudge warmers. Waffle cone irons usually need no exhaust hood: confirm it with your plan reviewer</t>
         </is>
       </c>
       <c r="E18" s="31" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="F10" s="28" t="inlineStr">
         <is>
-          <t>Share of total sales. Scoops, cups, cones and sundaes in the shop about 65%, hand-packed pints and quarts to go about 15%, ice cream cakes and holiday pies about 10%, catering about 5% and delivery marketplaces 4% (see "Delivery share of sales"). One sales tax rate in the example; in some states a packaged pint or a whole cake may be taxed as a grocery, so check your state</t>
+          <t>Share of total sales. Within this line, roughly: scoops, cups, cones and sundaes in the shop 65%, hand-packed pints and quarts to go 15%, ice cream cakes and holiday pies 10%, catering 5% and pints through delivery marketplaces the rest (see "Delivery share of total sales"). One sales tax rate in the example; in some states a packaged pint or a whole cake may be taxed as a grocery, so check your state</t>
         </is>
       </c>
       <c r="G10" s="67">
@@ -5813,7 +5813,7 @@
       </c>
       <c r="J7" s="28" t="inlineStr">
         <is>
-          <t>Seasonal part-time W-2 employee, about 40 hours a week from April to September, which equals half a full-time position over the year. Rehire each spring. Scoopers aged 14-15 only within the FLSA hours (29 CFR 570.35)</t>
+          <t>Seasonal W-2 employee: about 40 hours a week from April to September, which equals half a full-time position over the year (part-time on a yearly basis). Rehire each spring. Scoopers aged 14-15 only within the FLSA hours (29 CFR 570.35)</t>
         </is>
       </c>
     </row>
@@ -6465,7 +6465,7 @@
     <row r="8" ht="225" customHeight="1">
       <c r="A8" s="46" t="inlineStr">
         <is>
-          <t>4. All figures are shown EXCL. SALES TAX. To turn a menu price into a price without tax, divide it by 1 + your sales tax rate (8% in the example, so divide by 1.08). The scoop is taxed as prepared food; in some states packaged pints and whole cakes may be taxed as groceries, so check your state. The P&amp;L is excl. sales tax and the cash flow uses what is collected, tax included. Input tax on purchases is not recoverable in this book.</t>
+          <t>4. All figures are shown EXCL. SALES TAX. To turn a menu price into a price without tax, divide it by 1 + your sales tax rate (8% in the example, so divide by 1.08). A scoop is generally taxed as prepared food; in some states packaged pints and whole cakes may be taxed as groceries, so check your state. The P&amp;L is excl. sales tax and the cash flow uses what is collected, tax included. Input tax on purchases is not recoverable in this book.</t>
         </is>
       </c>
       <c r="B8" s="28" t="n"/>
@@ -6979,7 +6979,7 @@
       </c>
       <c r="B41" s="28" t="inlineStr">
         <is>
-          <t>Buying pasteurized base: retail license in most states; own mix: state dairy / frozen dessert manufacturer license</t>
+          <t>Buying pasteurized base: retail permit, plus a frozen dessert license in some states (Vermont); own mix: state dairy / frozen dessert manufacturer license</t>
         </is>
       </c>
       <c r="C41" s="28" t="inlineStr">
@@ -7978,7 +7978,7 @@
       </c>
       <c r="O13" s="28" t="inlineStr">
         <is>
-          <t>Twelve monthly payments, with no extra pay months unless you enter more than 12 pay periods on "0. Assumptions". The yearly total matches the P&amp;L. Payroll is spread over twelve months, but seasonal staff only get paid in season, so winter shows up more expensive and summer cheaper than reality: that is the prudent side. March and February barely change, but from June to January your real cash will be lower than on this tab (in the case, by about $10,000 in September)</t>
+          <t>Twelve monthly payments, with no extra pay months unless you enter more than 12 pay periods on "0. Assumptions". The yearly total matches the P&amp;L. Payroll is spread over twelve months, but seasonal staff only get paid in season, so winter shows up more expensive and summer cheaper than reality: that is the prudent side. March and February barely change, but from June to January your real cash will be lower than on this tab (in the case, by about $13,800 at the end of September)</t>
         </is>
       </c>
     </row>

</xml_diff>